<commit_message>
Fix Amount integer rounding and reject invalid configuration identities and ranges
</commit_message>
<xml_diff>
--- a/space-battleship/foundation/tests/excel/foundation.xlsx
+++ b/space-battleship/foundation/tests/excel/foundation.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -976,6 +976,106 @@
         </is>
       </c>
       <c r="I15" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>N01-floor-integer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>N01-ceil-integer</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ceil</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>N01-floor-adjacent</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>floor</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>112.9999999999</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>N01-ceil-adjacent</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ceil</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>109.0000000001</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>1e-12</v>
       </c>
     </row>

</xml_diff>